<commit_message>
补充 Moderna/BioNTech/Legend + 说明 PROTAC 归类
</commit_message>
<xml_diff>
--- a/公司x通路矩阵.xlsx
+++ b/公司x通路矩阵.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X41"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2916,43 +2916,161 @@
       <c r="W34" s="15" t="n"/>
       <c r="X34" s="15" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+    <row r="35" ht="47" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>补 Moderna · 🇺🇸 MRNA</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="15" t="n"/>
+      <c r="I35" s="15" t="n"/>
+      <c r="J35" s="15" t="n"/>
+      <c r="K35" s="15" t="n"/>
+      <c r="L35" s="15" t="n"/>
+      <c r="M35" s="15" t="n"/>
+      <c r="N35" s="15" t="n"/>
+      <c r="O35" s="15" t="n"/>
+      <c r="P35" s="15" t="n"/>
+      <c r="Q35" s="15" t="n"/>
+      <c r="R35" s="15" t="n"/>
+      <c r="S35" s="15" t="n"/>
+      <c r="T35" s="18" t="inlineStr">
+        <is>
+          <t>mRNA蛋白替代○</t>
+        </is>
+      </c>
+      <c r="U35" s="15" t="n"/>
+      <c r="V35" s="15" t="n"/>
+      <c r="W35" s="15" t="n"/>
+      <c r="X35" s="15" t="n"/>
+    </row>
+    <row r="36" ht="47" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>补 BioNTech · 🇩🇪 BNTX</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>PD-L1×VEGF双抗○</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>ADC/CAR-T○</t>
+        </is>
+      </c>
+      <c r="I36" s="15" t="n"/>
+      <c r="J36" s="15" t="n"/>
+      <c r="K36" s="15" t="n"/>
+      <c r="L36" s="15" t="n"/>
+      <c r="M36" s="15" t="n"/>
+      <c r="N36" s="15" t="n"/>
+      <c r="O36" s="15" t="n"/>
+      <c r="P36" s="15" t="n"/>
+      <c r="Q36" s="15" t="n"/>
+      <c r="R36" s="15" t="n"/>
+      <c r="S36" s="15" t="n"/>
+      <c r="T36" s="15" t="n"/>
+      <c r="U36" s="15" t="n"/>
+      <c r="V36" s="15" t="n"/>
+      <c r="W36" s="15" t="n"/>
+      <c r="X36" s="15" t="n"/>
+    </row>
+    <row r="37" ht="47" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>补 Legend Biotech · 🇺🇸 LEGN</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="003C6E64"/>
+              <sz val="9"/>
+            </rPr>
+            <t>1◆</t>
+          </r>
+        </is>
+      </c>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>BCMA CAR-T◆</t>
+        </is>
+      </c>
+      <c r="I37" s="15" t="n"/>
+      <c r="J37" s="15" t="n"/>
+      <c r="K37" s="15" t="n"/>
+      <c r="L37" s="15" t="n"/>
+      <c r="M37" s="15" t="n"/>
+      <c r="N37" s="15" t="n"/>
+      <c r="O37" s="15" t="n"/>
+      <c r="P37" s="15" t="n"/>
+      <c r="Q37" s="15" t="n"/>
+      <c r="R37" s="15" t="n"/>
+      <c r="S37" s="15" t="n"/>
+      <c r="T37" s="15" t="n"/>
+      <c r="U37" s="15" t="n"/>
+      <c r="V37" s="15" t="n"/>
+      <c r="W37" s="15" t="n"/>
+      <c r="X37" s="15" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>口径说明：</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="20" t="inlineStr">
-        <is>
-          <t>· 「★◆●计数」= 该公司在全部通路上 ★首创 / ◆领跑 / ●重要 的靶点数量合计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>· 每个格子里同一公司在该通路的多个靶点各自单独成行。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>· 红色加粗靶点 = 当下最热但尚未攻克/未成熟：KRAS(G12C/G12D/pan-RAS)、Lp(a)、amylin、DLL3、GPRC5D、Nav1.8。</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>· 仅标注有重大布局的靶点（非全管线）；不属于这些通路组的重磅（疫苗/HIV/抗凝/眼科VEGF/前列腺激素/EPO·G-CSF/骨·医美）见「公司词典」。</t>
+          <t>· 「★◆●计数」= 该公司在全部通路上 ★首创 / ◆领跑 / ●重要 的靶点数量合计。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>· 每个格子里同一公司在该通路的多个靶点各自单独成行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>· 红色加粗靶点 = 当下最热但尚未攻克/未成熟：KRAS(G12C/G12D/pan-RAS)、Lp(a)、amylin、DLL3、GPRC5D、Nav1.8。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>· 仅标注有重大布局的靶点（非全管线）；不属于这些通路组的重磅（疫苗/HIV/抗凝/眼科VEGF/前列腺激素/EPO·G-CSF/骨·医美）见「公司词典」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>· 已剔除非研发型：CVS(PBM)、WuXi(CRO)、Lonza(CDMO)；Sandoz为生物类似药商，整行留空。</t>
         </is>

</xml_diff>